<commit_message>
Bashful and Dopey switched DOAMIN_ID, now Bashful=3, Dopey=1
</commit_message>
<xml_diff>
--- a/hardware_test/test_results/summary/components_summary.xlsx
+++ b/hardware_test/test_results/summary/components_summary.xlsx
@@ -605,15 +605,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sleepy</t>
+          <t>Bashful</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2025-06-17T15:51:15</t>
+          <t>2025-06-14T12:27:58</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -681,29 +681,21 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No lidar; </t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Servo5 is loose</t>
-        </is>
-      </c>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Dopey</t>
+          <t>Sleepy</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2025-08-17T15:39:31</t>
+          <t>2025-06-17T15:51:15</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -713,24 +705,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>PASS</t>
@@ -773,15 +765,19 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Did not work with battery; </t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr"/>
+          <t xml:space="preserve">No lidar; </t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Servo5 is loose</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Bashful</t>
+          <t>Dopey</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -789,7 +785,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2025-06-14T12:27:58</t>
+          <t>2025-08-17T15:39:31</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -799,7 +795,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -857,11 +853,7 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Did not work with battery, died after ~5 minutes; </t>
-        </is>
-      </c>
+      <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
all 10 robots are good to go
</commit_message>
<xml_diff>
--- a/hardware_test/test_results/summary/components_summary.xlsx
+++ b/hardware_test/test_results/summary/components_summary.xlsx
@@ -531,7 +531,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2025-06-25T11:21:16</t>
+          <t>2025-12-21T13:04:44</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -613,7 +613,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2025-06-14T12:27:58</t>
+          <t>2025-11-22T12:27:58</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2025-06-17T15:51:15</t>
+          <t>2025-12-21T15:17:15</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -763,14 +763,10 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No lidar; </t>
-        </is>
-      </c>
+      <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Servo5 is loose</t>
+          <t>RGBD camera cable is missing</t>
         </is>
       </c>
     </row>
@@ -785,7 +781,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2025-08-17T15:39:31</t>
+          <t>2025-11-22T15:39:31</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -867,7 +863,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2025-08-17T11:30:23</t>
+          <t>2025-12-21T13:08:27</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -949,7 +945,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2025-06-12T17:22:05</t>
+          <t>2025-12-21T12:55:43</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1018,20 +1014,24 @@
         </is>
       </c>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>RGBD camera cable is missing</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Prince</t>
+          <t>Queen</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2025-06-27T14:31:47</t>
+          <t>2025-12-21T13:13:27</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1105,7 +1105,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SnowWhite</t>
+          <t>Snow</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2025-08-24T14:35:29</t>
+          <t>2025-12-21T12:46:19</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1182,24 +1182,20 @@
         </is>
       </c>
       <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>Electricity meter fixed</t>
-        </is>
-      </c>
+      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Queen</t>
+          <t>Huntsman</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2025-06-27T15:55:55</t>
+          <t>2025-12-21T13:21:54</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1281,7 +1277,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2025-06-13T11:24:15</t>
+          <t>2025-12-21T12:49:39</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">

</xml_diff>